<commit_message>
Strengthen v4 evidence with external execution and root concordance
</commit_message>
<xml_diff>
--- a/supplementary_tables/submission_v4/Plant_CellFM_Supplementary_Tables_v4.xlsx
+++ b/supplementary_tables/submission_v4/Plant_CellFM_Supplementary_Tables_v4.xlsx
@@ -22,6 +22,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S13_arabidopsis_root_marker_can" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S14_figure_and_source_data_mani" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S15_reproducibility_manifest.ts" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S16_arabidopsis_root_literature" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -13355,7 +13356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE9"/>
+  <dimension ref="A1:AF10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13512,6 +13513,11 @@
       <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>anonymous_api_accessible</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>audit_status</t>
         </is>
       </c>
     </row>
@@ -13587,6 +13593,7 @@
       <c r="AC2" t="inlineStr"/>
       <c r="AD2" t="inlineStr"/>
       <c r="AE2" t="inlineStr"/>
+      <c r="AF2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -13660,6 +13667,7 @@
       <c r="AC3" t="inlineStr"/>
       <c r="AD3" t="inlineStr"/>
       <c r="AE3" t="inlineStr"/>
+      <c r="AF3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -13733,6 +13741,7 @@
       <c r="AC4" t="inlineStr"/>
       <c r="AD4" t="inlineStr"/>
       <c r="AE4" t="inlineStr"/>
+      <c r="AF4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -13804,6 +13813,7 @@
       <c r="AC5" t="inlineStr"/>
       <c r="AD5" t="inlineStr"/>
       <c r="AE5" t="inlineStr"/>
+      <c r="AF5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -13875,6 +13885,7 @@
       <c r="AC6" t="inlineStr"/>
       <c r="AD6" t="inlineStr"/>
       <c r="AE6" t="inlineStr"/>
+      <c r="AF6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -13942,6 +13953,7 @@
       <c r="AC7" t="inlineStr"/>
       <c r="AD7" t="inlineStr"/>
       <c r="AE7" t="inlineStr"/>
+      <c r="AF7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -14011,6 +14023,7 @@
       <c r="AC8" t="inlineStr"/>
       <c r="AD8" t="inlineStr"/>
       <c r="AE8" t="inlineStr"/>
+      <c r="AF8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -14071,6 +14084,79 @@
       </c>
       <c r="AE9" t="b">
         <v>0</v>
+      </c>
+      <c r="AF9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>scPlantLLM official checkpoint execution on official processed chunks</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>official train/test chunks; stratified 256/256 frozen-encoder representation probe</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>completed_execution_not_matched_to_v17</t>
+        </is>
+      </c>
+      <c r="D10" t="b">
+        <v>0</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>release_metadata/scplantllm_official_execution_audit.json</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Official scPlantLLM weight execution passed the release audit with zero missing or unexpected state keys. Metric is a frozen-encoder centroid probe on scPlantLLM's own chunks, not the classifier head and not a matched Plant-CellFM v17 comparison.</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>scplantllm_frozen_embedding_nearest_centroid_probe</t>
+        </is>
+      </c>
+      <c r="Q10" t="n">
+        <v>256</v>
+      </c>
+      <c r="R10" t="n">
+        <v>256</v>
+      </c>
+      <c r="S10" t="n">
+        <v>0.83984375</v>
+      </c>
+      <c r="T10" t="n">
+        <v>0.8408133143539664</v>
+      </c>
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="inlineStr"/>
+      <c r="X10" t="inlineStr"/>
+      <c r="Y10" t="inlineStr"/>
+      <c r="Z10" t="inlineStr"/>
+      <c r="AA10" t="inlineStr"/>
+      <c r="AB10" t="inlineStr"/>
+      <c r="AC10" t="inlineStr"/>
+      <c r="AD10" t="inlineStr"/>
+      <c r="AE10" t="inlineStr"/>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -25575,7 +25661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25841,6 +25927,39 @@
         </is>
       </c>
       <c r="G8" t="inlineStr">
+        <is>
+          <t>600x600</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>extended_data</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>plant_cellfm_v4_ed_fig4_literature_marker_concordance</t>
+        </is>
+      </c>
+      <c r="C9" t="b">
+        <v>1</v>
+      </c>
+      <c r="D9" t="b">
+        <v>1</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>plant_cellfm_v4_ed_fig4_literature_marker_concordance_literature_marker_concordance.tsv; plant_cellfm_v4_ed_fig4_literature_marker_concordance_literature_marker_concordance_summary.tsv</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>4649x2314</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
         <is>
           <t>600x600</t>
         </is>
@@ -25857,7 +25976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25919,7 +26038,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ea83f3683043a57907f743a9de9c9f1ae65fbb2270f4137d16374365c5a263f2</t>
+          <t>4d1c063d3b66b74037b383b670c9df7951815548127511e97ac3f7c6d7892ab2</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -25931,86 +26050,522 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>scripts/write_submission_v4_supplementary_tables.py</t>
+          <t>scripts/build_v4_root_literature_concordance.py</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10163c907e09a0003dc32f320a9d9690a2347759a1693fe6f7a65011d376fb80</t>
+          <t>475c9e9b659002278d4903e73a3827c2f49b8940669d8d6e427e94ab603f8af3</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>python scripts/write_submission_v4_supplementary_tables.py</t>
+          <t>python scripts/build_v4_root_literature_concordance.py</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>scripts/audit_v4_submission_figure_suite.py</t>
+          <t>scripts/write_submission_v4_supplementary_tables.py</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ac001b5998140be2519834d7ed89154a8fa2154cc928fe778d973161d558877c</t>
+          <t>a5d9377dd1ed672d12ef34a00352e5a6b953047365d038672e0de35e2fecd086</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>python scripts/audit_v4_submission_figure_suite.py</t>
+          <t>python scripts/write_submission_v4_supplementary_tables.py</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>release_metadata/revision_v17_nested_metadata_gate.json</t>
+          <t>scripts/audit_v4_submission_figure_suite.py</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>349161e42cff619b5aed2bba6e73eacf04cc5706549ef60e26b73ea08a46e5bb</t>
+          <t>affa0beffeb4b4ad49098d767764238aa8373dc724125314c4e32a3876343f2b</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>frozen release record</t>
+          <t>python scripts/audit_v4_submission_figure_suite.py</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>release_metadata/revision_v18_identity_curated_strict.json</t>
+          <t>scripts/audit_scplantllm_official_execution.py</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ecc55ce802fb8bfa15ecb684bf24a216d087adcc8a5892cb218f998cf02a6242</t>
+          <t>79851d3c34781731f3ca32ffc81b356ee10bcae8e817145a14d72b6d52b8228f</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>frozen release record</t>
+          <t>python scripts/audit_scplantllm_official_execution.py</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>release_metadata/revision_v17_nested_metadata_gate.json</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>349161e42cff619b5aed2bba6e73eacf04cc5706549ef60e26b73ea08a46e5bb</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>frozen release record</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>release_metadata/revision_v18_identity_curated_strict.json</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ecc55ce802fb8bfa15ecb684bf24a216d087adcc8a5892cb218f998cf02a6242</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>frozen release record</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>release_metadata/plant_cellfm_model_card_v4.json</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>3f743d8cd288133a402e24b499377611273d516e3a213dae488697ca61909deb</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>8805d5ae2c5488af181ef64817bec8b30eadcf9aa79fa5c1e144b751f69e8e17</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
         <is>
           <t>frozen release record</t>
         </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>release_metadata/scplantllm_official_data_embedding_probe_256.json</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>30fb56f75e0f10bcbff682f6dd95a326852f28ccae0e9abfb438377191af3238</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>frozen release record</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>release_metadata/scplantllm_official_execution_audit.json</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>7168a231a1fa50e114f60d1b8abd9d3d606c530f4d10d3e54903b386672a8bd9</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>frozen release record</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>release_metadata/arabidopsis_root_literature_concordance_v4.json</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>8889f0b663f8959b8fb786bf7228ef77d84504cd81ccf77b6d654055729c7d20</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>frozen release record</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>label</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>marker_symbol</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>gene</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>literature_identity</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>source_key</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>candidate_top_n</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>recovered_in_matching_program</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>candidate_rank</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>candidate_score</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>candidate_log2fc</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>candidate_detection_in</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>candidate_detection_out</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>candidate_detection_delta</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Root hair</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>COBL9</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>AT5G49270</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>root-hair epidermis</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>jean_baptiste_2019</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>20</v>
+      </c>
+      <c r="G2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Non-hair</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>WER</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>AT5G14750</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>non-hair / atrichoblast epidermis</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>jean_baptiste_2019</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>20</v>
+      </c>
+      <c r="G3" t="b">
+        <v>0</v>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Non-hair</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>GL2</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>AT1G79840</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>non-hair / atrichoblast epidermis</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>jean_baptiste_2019</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>20</v>
+      </c>
+      <c r="G4" t="b">
+        <v>0</v>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Root endodermis</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>CASP1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>AT2G36100</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>endodermis</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>shahan_2022</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>20</v>
+      </c>
+      <c r="G5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H5" t="n">
+        <v>7</v>
+      </c>
+      <c r="I5" t="n">
+        <v>2.394655227661133</v>
+      </c>
+      <c r="J5" t="n">
+        <v>4.255702018737793</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.6027033925056458</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.0400100350379943</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.5626933574676515</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Phloem</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>APL</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>AT1G79430</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>phloem within the stele</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>jean_baptiste_2019</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>20</v>
+      </c>
+      <c r="G6" t="b">
+        <v>1</v>
+      </c>
+      <c r="H6" t="n">
+        <v>4</v>
+      </c>
+      <c r="I6" t="n">
+        <v>2.545392036437988</v>
+      </c>
+      <c r="J6" t="n">
+        <v>7.071040630340576</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.3624161183834076</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.0024419331457465</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.3599741852376611</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Xylem</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>MYB46</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>AT5G12870</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>xylem within the stele</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>jean_baptiste_2019</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>20</v>
+      </c>
+      <c r="G7" t="b">
+        <v>1</v>
+      </c>
+      <c r="H7" t="n">
+        <v>12</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1.641520142555237</v>
+      </c>
+      <c r="J7" t="n">
+        <v>7.205848217010498</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.2292609363794326</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.001457059639506</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.2278038767399266</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add external root evidence and submission visuals
</commit_message>
<xml_diff>
--- a/supplementary_tables/submission_v4/Plant_CellFM_Supplementary_Tables_v4.xlsx
+++ b/supplementary_tables/submission_v4/Plant_CellFM_Supplementary_Tables_v4.xlsx
@@ -23,6 +23,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S14_figure_and_source_data_mani" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S15_reproducibility_manifest.ts" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S16_arabidopsis_root_literature" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S17_gse152766_external_root_bli" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25661,7 +25662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25960,6 +25961,39 @@
         </is>
       </c>
       <c r="G9" t="inlineStr">
+        <is>
+          <t>600x600</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>extended_data</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>plant_cellfm_v4_ed_fig5_external_root_blind_inference</t>
+        </is>
+      </c>
+      <c r="C10" t="b">
+        <v>1</v>
+      </c>
+      <c r="D10" t="b">
+        <v>1</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>plant_cellfm_v4_ed_fig5_external_root_blind_inference_external_embedding_umap.tsv; plant_cellfm_v4_ed_fig5_external_root_blind_inference_external_marker_coherence.tsv; plant_cellfm_v4_ed_fig5_external_root_blind_inference_external_prediction_distribution.tsv</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>4679x4152</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
         <is>
           <t>600x600</t>
         </is>
@@ -25976,7 +26010,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26038,7 +26072,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>4d1c063d3b66b74037b383b670c9df7951815548127511e97ac3f7c6d7892ab2</t>
+          <t>f64a8cf64ccd65605bbb5f48f58e1ec308825583060a6ac353d1bf8c815bb578</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -26067,114 +26101,114 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>scripts/write_submission_v4_supplementary_tables.py</t>
+          <t>scripts/download_gse152766_external_root_case.py</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>a5d9377dd1ed672d12ef34a00352e5a6b953047365d038672e0de35e2fecd086</t>
+          <t>83df87e66ba9037d186099ac8ed8cbf1fe4f6cdabdfa4d7d21960b07a5a0e02e</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>python scripts/write_submission_v4_supplementary_tables.py</t>
+          <t>python scripts/download_gse152766_external_root_case.py</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>scripts/audit_v4_submission_figure_suite.py</t>
+          <t>scripts/prepare_gse152766_external_root_case.py</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>affa0beffeb4b4ad49098d767764238aa8373dc724125314c4e32a3876343f2b</t>
+          <t>74e7b2a4c448bdf3cc7b308745b26e74a4f6b0d0aabba2c265259a14705ac4c6</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>python scripts/audit_v4_submission_figure_suite.py</t>
+          <t>python scripts/prepare_gse152766_external_root_case.py</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>scripts/audit_scplantllm_official_execution.py</t>
+          <t>scripts/audit_gse152766_external_root_case.py</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>79851d3c34781731f3ca32ffc81b356ee10bcae8e817145a14d72b6d52b8228f</t>
+          <t>e53fe0a5c7d8da4db2d531d307840a4ad116681d6705e907ee42b5c30c89a55d</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>python scripts/audit_scplantllm_official_execution.py</t>
+          <t>python scripts/audit_gse152766_external_root_case.py</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>release_metadata/revision_v17_nested_metadata_gate.json</t>
+          <t>scripts/write_submission_v4_supplementary_tables.py</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>349161e42cff619b5aed2bba6e73eacf04cc5706549ef60e26b73ea08a46e5bb</t>
+          <t>cd4f63dd27fc08a815b9b450566db25a5ddb9f976510a89d0e7de372c1981393</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>frozen release record</t>
+          <t>python scripts/write_submission_v4_supplementary_tables.py</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>release_metadata/revision_v18_identity_curated_strict.json</t>
+          <t>scripts/audit_v4_submission_figure_suite.py</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ecc55ce802fb8bfa15ecb684bf24a216d087adcc8a5892cb218f998cf02a6242</t>
+          <t>95ca1cc65f4535a06bb6271e0a833735c85e68552b9f30c5bd3e328fd7621e81</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>frozen release record</t>
+          <t>python scripts/audit_v4_submission_figure_suite.py</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>release_metadata/plant_cellfm_model_card_v4.json</t>
+          <t>scripts/audit_scplantllm_official_execution.py</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>8805d5ae2c5488af181ef64817bec8b30eadcf9aa79fa5c1e144b751f69e8e17</t>
+          <t>79851d3c34781731f3ca32ffc81b356ee10bcae8e817145a14d72b6d52b8228f</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>frozen release record</t>
+          <t>python scripts/audit_scplantllm_official_execution.py</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>release_metadata/scplantllm_official_data_embedding_probe_256.json</t>
+          <t>release_metadata/revision_v17_nested_metadata_gate.json</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>30fb56f75e0f10bcbff682f6dd95a326852f28ccae0e9abfb438377191af3238</t>
+          <t>349161e42cff619b5aed2bba6e73eacf04cc5706549ef60e26b73ea08a46e5bb</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -26186,12 +26220,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>release_metadata/scplantllm_official_execution_audit.json</t>
+          <t>release_metadata/revision_v18_identity_curated_strict.json</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>7168a231a1fa50e114f60d1b8abd9d3d606c530f4d10d3e54903b386672a8bd9</t>
+          <t>ecc55ce802fb8bfa15ecb684bf24a216d087adcc8a5892cb218f998cf02a6242</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -26203,15 +26237,100 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>release_metadata/plant_cellfm_model_card_v4.json</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>49acbebcc5f8e9b9a2edc1a3c5160c40cda1df2f3a0ffdb6c3eb83563e01cc03</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>frozen release record</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>release_metadata/scplantllm_official_data_embedding_probe_256.json</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>30fb56f75e0f10bcbff682f6dd95a326852f28ccae0e9abfb438377191af3238</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>frozen release record</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>release_metadata/scplantllm_official_execution_audit.json</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>7168a231a1fa50e114f60d1b8abd9d3d606c530f4d10d3e54903b386672a8bd9</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>frozen release record</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>release_metadata/arabidopsis_root_literature_concordance_v4.json</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>8889f0b663f8959b8fb786bf7228ef77d84504cd81ccf77b6d654055729c7d20</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>frozen release record</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>release_metadata/gse152766_external_input_acquisition_v4.json</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>e13d7b97131df7ee4b1af9f0989f8653ca3bc774019c0b830239540f6196b632</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>frozen release record</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>release_metadata/gse152766_external_root_blind_inference_v4.json</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>c48020926be71aa8d5e063c71449902cd499710a3999e0c5e8eb3b560d19a6e5</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
         <is>
           <t>frozen release record</t>
         </is>
@@ -26573,6 +26692,427 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>expected_label</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>marker_symbol</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>gene_id</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>literature_key</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>predicted_label_cells</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>target_mean_log1p_normalised_expression</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>outside_mean_log1p_normalised_expression</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>mean_expression_delta</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>target_detection_fraction</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>outside_detection_fraction</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>detection_fraction_delta</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>rank_among_predicted_labels_by_mean_expression</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>rank_among_predicted_labels_by_detection_fraction</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>is_top_mean_expression_label</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>is_top_detection_label</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Root hair</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>COBL9</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>AT5G49270</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>jean_baptiste_2019</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>168</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.7595265883414269</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.04519819918830953</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.7143283891531174</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.6726190476190477</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.05032822757111598</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.6222908200479317</v>
+      </c>
+      <c r="L2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N2" t="b">
+        <v>1</v>
+      </c>
+      <c r="O2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Non-hair</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>WER</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>AT5G14750</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>jean_baptiste_2019</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>428</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.07833718756583632</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.06001101661122948</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.01832617095460684</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.1588785046728972</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.08145975887911372</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.07741874579378347</v>
+      </c>
+      <c r="L3" t="n">
+        <v>4</v>
+      </c>
+      <c r="M3" t="n">
+        <v>3</v>
+      </c>
+      <c r="N3" t="b">
+        <v>0</v>
+      </c>
+      <c r="O3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Non-hair</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>GL2</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>AT1G79840</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>jean_baptiste_2019</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>428</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.1616766836788782</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.03053287187659477</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.1311438118022835</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.2383177570093458</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.05555555555555555</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.1827622014537902</v>
+      </c>
+      <c r="L4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N4" t="b">
+        <v>1</v>
+      </c>
+      <c r="O4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Root endodermis</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>CASP1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>AT2G36100</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>shahan_2022</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>321</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.0836947109930169</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.00180918886331487</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.08188552212970203</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.02180685358255452</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.001281024819855885</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.02052582876269863</v>
+      </c>
+      <c r="L5" t="n">
+        <v>1</v>
+      </c>
+      <c r="M5" t="n">
+        <v>1</v>
+      </c>
+      <c r="N5" t="b">
+        <v>1</v>
+      </c>
+      <c r="O5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Phloem</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>APL</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>AT1G79430</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>jean_baptiste_2019</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1.012643594738103</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.005530055345931204</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1.007113539392172</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.003200243828101189</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.7467997561718989</v>
+      </c>
+      <c r="L6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N6" t="b">
+        <v>1</v>
+      </c>
+      <c r="O6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Xylem</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>MYB46</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>AT5G12870</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>jean_baptiste_2019</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>191</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.02820420641642984</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.003050878514996647</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.02515332790143319</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.02617801047120419</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.002823529411764706</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.02335448105943948</v>
+      </c>
+      <c r="L7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N7" t="b">
+        <v>1</v>
+      </c>
+      <c r="O7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
release: add wheat adaptation and submission figure package
</commit_message>
<xml_diff>
--- a/supplementary_tables/submission_v4/Plant_CellFM_Supplementary_Tables_v4.xlsx
+++ b/supplementary_tables/submission_v4/Plant_CellFM_Supplementary_Tables_v4.xlsx
@@ -24,6 +24,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S15_reproducibility_manifest.ts" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S16_arabidopsis_root_literature" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S17_gse152766_external_root_bli" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S18_GSE270140_secondary_root_ad" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S19_GSE270140_secondary_root_ad" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S20_GSE270342_wheat_root_adapte" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26010,7 +26013,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26152,114 +26155,114 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>scripts/write_submission_v4_supplementary_tables.py</t>
+          <t>scripts/prepare_gse270342_wheat_root_case.py</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>cd4f63dd27fc08a815b9b450566db25a5ddb9f976510a89d0e7de372c1981393</t>
+          <t>9deedf597f31807be50930fd8437bfec632ce95c718be8e819a9b267d111382a</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>python scripts/write_submission_v4_supplementary_tables.py</t>
+          <t>python scripts/prepare_gse270342_wheat_root_case.py</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>scripts/audit_v4_submission_figure_suite.py</t>
+          <t>scripts/audit_gse270342_wheat_lora_adapter.py</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>95ca1cc65f4535a06bb6271e0a833735c85e68552b9f30c5bd3e328fd7621e81</t>
+          <t>ed1215964424a5da6fefa6dea71b0a75492c4a9ee99a6821c19ff5d2410a012d</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>python scripts/audit_v4_submission_figure_suite.py</t>
+          <t>python scripts/audit_gse270342_wheat_lora_adapter.py</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>scripts/audit_scplantllm_official_execution.py</t>
+          <t>scripts/render_v5_wheat_root_adapter_figure.py</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>79851d3c34781731f3ca32ffc81b356ee10bcae8e817145a14d72b6d52b8228f</t>
+          <t>927f58140cc9fc0c17bc2944982caa90fdd04526ef2478c396ca8b16798f3311</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>python scripts/audit_scplantllm_official_execution.py</t>
+          <t>python scripts/render_v5_wheat_root_adapter_figure.py</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>release_metadata/revision_v17_nested_metadata_gate.json</t>
+          <t>scripts/write_submission_v4_supplementary_tables.py</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>349161e42cff619b5aed2bba6e73eacf04cc5706549ef60e26b73ea08a46e5bb</t>
+          <t>3d07b6219dcac8381d3edd2211e4c708182efbc569b47c198a18a1a63381e11a</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>frozen release record</t>
+          <t>python scripts/write_submission_v4_supplementary_tables.py</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>release_metadata/revision_v18_identity_curated_strict.json</t>
+          <t>scripts/audit_v4_submission_figure_suite.py</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ecc55ce802fb8bfa15ecb684bf24a216d087adcc8a5892cb218f998cf02a6242</t>
+          <t>95ca1cc65f4535a06bb6271e0a833735c85e68552b9f30c5bd3e328fd7621e81</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>frozen release record</t>
+          <t>python scripts/audit_v4_submission_figure_suite.py</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>release_metadata/plant_cellfm_model_card_v4.json</t>
+          <t>scripts/audit_scplantllm_official_execution.py</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>49acbebcc5f8e9b9a2edc1a3c5160c40cda1df2f3a0ffdb6c3eb83563e01cc03</t>
+          <t>79851d3c34781731f3ca32ffc81b356ee10bcae8e817145a14d72b6d52b8228f</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>frozen release record</t>
+          <t>python scripts/audit_scplantllm_official_execution.py</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>release_metadata/scplantllm_official_data_embedding_probe_256.json</t>
+          <t>release_metadata/revision_v17_nested_metadata_gate.json</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>30fb56f75e0f10bcbff682f6dd95a326852f28ccae0e9abfb438377191af3238</t>
+          <t>349161e42cff619b5aed2bba6e73eacf04cc5706549ef60e26b73ea08a46e5bb</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -26271,12 +26274,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>release_metadata/scplantllm_official_execution_audit.json</t>
+          <t>release_metadata/revision_v18_identity_curated_strict.json</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>7168a231a1fa50e114f60d1b8abd9d3d606c530f4d10d3e54903b386672a8bd9</t>
+          <t>ecc55ce802fb8bfa15ecb684bf24a216d087adcc8a5892cb218f998cf02a6242</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -26288,12 +26291,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>release_metadata/arabidopsis_root_literature_concordance_v4.json</t>
+          <t>release_metadata/plant_cellfm_model_card_v4.json</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>8889f0b663f8959b8fb786bf7228ef77d84504cd81ccf77b6d654055729c7d20</t>
+          <t>aa6afc94a6a14d6527a68602b9b18dccc3f3a028eda7569ca990c9353daf844a</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -26305,12 +26308,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>release_metadata/gse152766_external_input_acquisition_v4.json</t>
+          <t>release_metadata/scplantllm_official_data_embedding_probe_256.json</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>e13d7b97131df7ee4b1af9f0989f8653ca3bc774019c0b830239540f6196b632</t>
+          <t>30fb56f75e0f10bcbff682f6dd95a326852f28ccae0e9abfb438377191af3238</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -26322,15 +26325,117 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>release_metadata/scplantllm_official_execution_audit.json</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>7168a231a1fa50e114f60d1b8abd9d3d606c530f4d10d3e54903b386672a8bd9</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>frozen release record</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>release_metadata/arabidopsis_root_literature_concordance_v4.json</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>8889f0b663f8959b8fb786bf7228ef77d84504cd81ccf77b6d654055729c7d20</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>frozen release record</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>release_metadata/gse152766_external_input_acquisition_v4.json</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>e13d7b97131df7ee4b1af9f0989f8653ca3bc774019c0b830239540f6196b632</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>frozen release record</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>release_metadata/gse152766_external_root_blind_inference_v4.json</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>c48020926be71aa8d5e063c71449902cd499710a3999e0c5e8eb3b560d19a6e5</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>frozen release record</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>release_metadata/gse270140_secondary_root_adapter_audit_v1.json</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>9a128dd31b5d741746c6cc3e176d65e2c912b6354cfd6b7b5f9d40e5d2770ee6</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>frozen release record</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>release_metadata/gse270342_wheat_nonoverlap_input_preparation_v1.json</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>81b5012bbff468efda2fd242bb4c1c15574d8f440ed206a86526c04e92b67ea3</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>frozen release record</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>release_metadata/gse270342_wheat_lora_adapter_audit_v1.json</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ab888b6c7a33a1c4390b6888be10510b3e0fa8a705fc434807c02352cfb824ad</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
         <is>
           <t>frozen release record</t>
         </is>
@@ -27113,6 +27218,392 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>author_annotation</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>support</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>precision</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>f1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Mature phloem parenchyma</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>645</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.8879456706281834</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.8108527131782945</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.8476499189627229</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Periderm</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>436</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.8957816377171216</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.8279816513761468</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.8605482717520858</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Vascular cambium</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>355</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.8828571428571429</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.8704225352112676</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.8765957446808511</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Conductive phloem parenchyma</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>247</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.6830985915492958</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.7854251012145749</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.7306967984934086</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Maturing xylem parenchyma</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>164</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.8957055214723927</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.8902439024390244</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.8929663608562691</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Young xylem parenchyma</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>148</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.8289473684210527</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.8513513513513513</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.84</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Mature xylem parenchyma</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>123</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.8111888111888111</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.943089430894309</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.8721804511278195</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Fiber</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>111</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.7606837606837606</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.8018018018018018</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.7807017543859649</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Companion cell</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>30</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.8787878787878788</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.9666666666666667</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.9206349206349206</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Vessel identity cell/expanding vessel</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>30</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.6222222222222222</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.9333333333333333</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.7466666666666667</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Myrosin idioblasts</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>24</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.9230769230769231</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Sieve element</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>23</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.7241379310344828</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.9130434782608695</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.8076923076923077</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Late differentiating vessel</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>9</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.7777777777777778</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.875</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Lateral root primordium/meristem</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>7</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.7777777777777778</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.875</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>method</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>cells</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>accuracy</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>macro_f1</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>weighted_f1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Frozen base checkpoint</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1885</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.02015915119363395</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.06033360236750066</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.03490112459136421</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Secondary-root LoRA-mode adapter</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1885</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.9092838196286472</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.9158917450162316</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.9204987447241185</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -27341,6 +27832,580 @@
       <c r="I6" t="inlineStr">
         <is>
           <t>deployment analysis; not strict zero-shot</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>interpretation</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Source and provenance</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>GEO series</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>GSE270342</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>accession</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>public author-labelled wheat root study</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Source and provenance</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Publication DOI</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>10.1016/j.celrep.2025.115240</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>DOI</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>source publication</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Source and provenance</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Author object cells</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>7388</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>cells</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>before overlap exclusion</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Source and provenance</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Historical strict-transfer rows</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>256</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>rows</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>recorded exploratory subset</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Source and provenance</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Exact CS1 barcodes excluded</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>224</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>cells</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>removed before inference and tuning</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Source and provenance</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Retained non-overlap cells</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>7164</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>cells</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>author-labelled same-study adaptation input</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Orthogroup mapping</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Source genes</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>78115</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>features</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>author object RNA count matrix</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Orthogroup mapping</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Checkpoint-compatible mapped genes</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>41987</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>features</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>mapped into frozen checkpoint vocabulary</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Orthogroup mapping</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Checkpoint-compatible feature fraction</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0.5375024003072393</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>fraction</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>feature-level mapping coverage</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Orthogroup mapping</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Checkpoint-compatible UMI fraction</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0.7632529502682207</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>fraction</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>count-weighted mapping coverage</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Locked split</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Train cells</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>5014</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>cells</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>fixed group-random split; seed 20260801</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Locked split</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Validation cells</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>717</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>cells</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>used for epoch selection</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Locked split</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Test cells</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1433</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>cells</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>locked author-label-supervised report</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Locked 13-class report</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>0.6224703419399861</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>fraction</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>full author-label test denominator</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Locked 13-class report</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Macro-F1</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0.6660112830533416</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>fraction</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>13 author labels</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Matched direct-root diagnostic</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Comparable cells</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>964</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>cells</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>predeclared eight-label map only</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Matched direct-root diagnostic</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Frozen first-projection accuracy</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>0.2593360995850623</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>fraction</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>frozen diagnostic, not the 13-class report</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Matched direct-root diagnostic</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>LoRA adapter accuracy</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>0.5622406639004149</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>fraction</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>same matched cells and mapping</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Matched direct-root diagnostic</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Accuracy gain</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>30.29045643153527</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>percentage points</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>adapted minus frozen</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Release identity</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Released adapter SHA256</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>597b7e425b0355ddfa81e4f5c9c63e85987d6b72fe49a841736b200ea6c2c22e</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>SHA256</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>models/Plant_CellFM_GSE270342_wheat_root_lora_adapter_best.pt</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Claim boundary</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Interpretation</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>The adapter is evaluated on a fixed, author-label-supervised cell-level test split from a public wheat root study after excluding exact barcode overlap with a prior strict-transfer subset. It is not a zero-shot or independent external validation result. The matched direct-root comparison is restricted to the predeclared eight-label map and does not replace the full 13-class author-label test metric.</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>not zero-shot, independent external validation or a third-party ranking</t>
         </is>
       </c>
     </row>

</xml_diff>